<commit_message>
Finish debugging and update tests
</commit_message>
<xml_diff>
--- a/analysis/Documentation/Analysis workflow.xlsx
+++ b/analysis/Documentation/Analysis workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\analysis\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F222047-D56B-45C8-B24F-9EA4CDD0FBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1002FBF-50C6-4185-BFB8-09EB4B237615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="360" windowWidth="15540" windowHeight="15120" xr2:uid="{DA17B847-4E6F-4D74-B79D-451C7E8DB918}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>Notebook cell 3</t>
   </si>
@@ -162,6 +162,33 @@
   </si>
   <si>
     <t>session=rebuild_and_validate_signals_registry</t>
+  </si>
+  <si>
+    <t>dt = infer_dt</t>
+  </si>
+  <si>
+    <t>target_cols = pick_cols</t>
+  </si>
+  <si>
+    <t>pick numeric cols to process (seems a bit dumb)</t>
+  </si>
+  <si>
+    <t>out=df.copy</t>
+  </si>
+  <si>
+    <t>data = ().interpolate</t>
+  </si>
+  <si>
+    <t>loop through target_cols:</t>
+  </si>
+  <si>
+    <t>out(vel_col)</t>
+  </si>
+  <si>
+    <t>out(acc_col)</t>
+  </si>
+  <si>
+    <t>va.py</t>
   </si>
 </sst>
 </file>
@@ -541,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{912255E3-2284-4ECE-B687-7253785F39DB}">
-  <dimension ref="A3:O48"/>
+  <dimension ref="A3:O53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -630,142 +657,183 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E28" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>43</v>
+      </c>
+      <c r="O24" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E29" t="s">
+    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E30" t="s">
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E31" t="s">
+    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E32" t="s">
+    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E37" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E33" t="s">
+    <row r="38" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D34" t="s">
+    <row r="39" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D35" t="s">
+    <row r="40" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D36" t="s">
+    <row r="41" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D37" t="s">
+    <row r="42" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D38" t="s">
+    <row r="43" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E39" t="s">
+    <row r="44" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E44" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E40" t="s">
+    <row r="45" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E45" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E41" t="s">
+    <row r="46" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E46" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F42" t="s">
+    <row r="47" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F47" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E43" t="s">
+    <row r="48" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E48" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D44" t="s">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D45" t="s">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>0</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B52" t="s">
         <v>18</v>
       </c>
-      <c r="O47" s="1" t="s">
+      <c r="O52" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>0</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B53" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add global strict / tolerant flag to data ingestion pipeline
</commit_message>
<xml_diff>
--- a/analysis/Documentation/Analysis workflow.xlsx
+++ b/analysis/Documentation/Analysis workflow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\analysis\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1002FBF-50C6-4185-BFB8-09EB4B237615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D1C5A-B692-4E23-9457-116CA52F0B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="360" windowWidth="15540" windowHeight="15120" xr2:uid="{DA17B847-4E6F-4D74-B79D-451C7E8DB918}"/>
+    <workbookView xWindow="3180" yWindow="105" windowWidth="32070" windowHeight="15120" xr2:uid="{DA17B847-4E6F-4D74-B79D-451C7E8DB918}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>Notebook cell 3</t>
   </si>
@@ -189,6 +189,15 @@
   </si>
   <si>
     <t>va.py</t>
+  </si>
+  <si>
+    <t>event_def = _schema_event_def_for_bundle</t>
+  </si>
+  <si>
+    <t>metric_specs = event_def.get("metrics")</t>
+  </si>
+  <si>
+    <t>loop through spec in metric_specs:</t>
   </si>
 </sst>
 </file>
@@ -568,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{912255E3-2284-4ECE-B687-7253785F39DB}">
-  <dimension ref="A3:O53"/>
+  <dimension ref="A3:O58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -800,40 +809,50 @@
     </row>
     <row r="47" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F47" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D49" t="s">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D50" t="s">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D55" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>0</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B57" t="s">
         <v>18</v>
       </c>
-      <c r="O52" s="1" t="s">
+      <c r="O57" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>0</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B58" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>